<commit_message>
feat(api-test): implement and verify Phase 2 keyword-driven API tests
</commit_message>
<xml_diff>
--- a/data/justkept/api/justkept_api_test_cases.xlsx
+++ b/data/justkept/api/justkept_api_test_cases.xlsx
@@ -21,8 +21,9 @@
     <sheet name="Broker_CreateDocumentDraft" sheetId="16" r:id="rId16"/>
     <sheet name="Document_FindRequestByReqId" sheetId="17" r:id="rId17"/>
     <sheet name="Broker_ListScheduleDraft" sheetId="18" r:id="rId18"/>
-    <sheet name="Broker_CustomerLogs" sheetId="19" r:id="rId19"/>
-    <sheet name="Broker_FindAllCusBySubComId" sheetId="20" r:id="rId20"/>
+    <sheet name="Audit_FindAuditLogs" sheetId="19" r:id="rId19"/>
+    <sheet name="Broker_CustomerLogs" sheetId="20" r:id="rId20"/>
+    <sheet name="Broker_FindAllCusBySubComId" sheetId="21" r:id="rId21"/>
   </sheets>
 </workbook>
 </file>
@@ -440,7 +441,7 @@
         <v>SET_BASE_URL</v>
       </c>
       <c r="C2" t="str">
-        <v>https://justkept-dev.freewillsolutions.com</v>
+        <v>justkept-dev.freewillsolutions.com</v>
       </c>
     </row>
     <row r="3">
@@ -547,7 +548,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:D7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -571,7 +572,7 @@
         <v>SET_BASE_URL</v>
       </c>
       <c r="C2" t="str">
-        <v>https://justkept-dev.freewillsolutions.com</v>
+        <v>justkept-dev.freewillsolutions.com</v>
       </c>
     </row>
     <row r="3">
@@ -610,10 +611,10 @@
         <v>API_POST</v>
       </c>
       <c r="C5" t="str">
-        <v>/api/broker/findallcustomerbysubcomid</v>
+        <v>/api/broker/findallcustomerbybrokerid</v>
       </c>
       <c r="D5" t="str">
-        <v>{"brokerId":"U1001", "cardId": "1100100123456"}</v>
+        <v>{"brokerId":"U1001"}</v>
       </c>
     </row>
     <row r="6">
@@ -624,7 +625,7 @@
         <v>LOG_RESPONSE</v>
       </c>
       <c r="C6" t="str">
-        <v>1500</v>
+        <v>500</v>
       </c>
     </row>
     <row r="7">
@@ -641,170 +642,16 @@
         <v>pass</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8">
-        <v>7</v>
-      </c>
-      <c r="B8" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C8" t="str">
-        <v>0.ID_Number|1100100123456</v>
-      </c>
-      <c r="D8" t="str">
-        <v>pass</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9">
-        <v>8</v>
-      </c>
-      <c r="B9" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C9" t="str">
-        <v>0.entity|relationship</v>
-      </c>
-      <c r="D9" t="str">
-        <v>pass</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10">
-        <v>9</v>
-      </c>
-      <c r="B10" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C10" t="str">
-        <v>0.PK|customer_relationship</v>
-      </c>
-      <c r="D10" t="str">
-        <v>pass</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11">
-        <v>10</v>
-      </c>
-      <c r="B11" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C11" t="str">
-        <v>0.customerIdGSIPK|undefined</v>
-      </c>
-      <c r="D11" t="str">
-        <v>fail</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12">
-        <v>11</v>
-      </c>
-      <c r="B12" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C12" t="str">
-        <v>0.customerName|undefined</v>
-      </c>
-      <c r="D12" t="str">
-        <v>fail</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13">
-        <v>12</v>
-      </c>
-      <c r="B13" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C13" t="str">
-        <v>0.email|undefined</v>
-      </c>
-      <c r="D13" t="str">
-        <v>fail</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14">
-        <v>13</v>
-      </c>
-      <c r="B14" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C14" t="str">
-        <v>0.pendingReq|undefined</v>
-      </c>
-      <c r="D14" t="str">
-        <v>fail</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15">
-        <v>14</v>
-      </c>
-      <c r="B15" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C15" t="str">
-        <v>0.status|undefined</v>
-      </c>
-      <c r="D15" t="str">
-        <v>fail</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16">
-        <v>15</v>
-      </c>
-      <c r="B16" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C16" t="str">
-        <v>0.subCompanyId|undefined</v>
-      </c>
-      <c r="D16" t="str">
-        <v>fail</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17">
-        <v>16</v>
-      </c>
-      <c r="B17" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C17" t="str">
-        <v>0.totalDocuments|undefined</v>
-      </c>
-      <c r="D17" t="str">
-        <v>fail</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18">
-        <v>17</v>
-      </c>
-      <c r="B18" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C18" t="str">
-        <v>0.updatedAt|undefined</v>
-      </c>
-      <c r="D18" t="str">
-        <v>fail</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D18"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D7"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -828,7 +675,7 @@
         <v>SET_BASE_URL</v>
       </c>
       <c r="C2" t="str">
-        <v>https://justkept-dev.freewillsolutions.com</v>
+        <v>justkept-dev.freewillsolutions.com</v>
       </c>
     </row>
     <row r="3">
@@ -881,7 +728,7 @@
         <v>LOG_RESPONSE</v>
       </c>
       <c r="C6" t="str">
-        <v>1500</v>
+        <v>500</v>
       </c>
     </row>
     <row r="7">
@@ -898,72 +745,16 @@
         <v>pass</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8">
-        <v>7</v>
-      </c>
-      <c r="B8" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C8" t="str">
-        <v>items.0.subCompanyId|BKK01</v>
-      </c>
-      <c r="D8" t="str">
-        <v>pass</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9">
-        <v>8</v>
-      </c>
-      <c r="B9" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C9" t="str">
-        <v>items.0.entity|customer_req</v>
-      </c>
-      <c r="D9" t="str">
-        <v>pass</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10">
-        <v>9</v>
-      </c>
-      <c r="B10" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C10" t="str">
-        <v>items.0.requestId|undefined</v>
-      </c>
-      <c r="D10" t="str">
-        <v>fail</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11">
-        <v>10</v>
-      </c>
-      <c r="B11" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C11" t="str">
-        <v>items.0.requestTopic|undefined</v>
-      </c>
-      <c r="D11" t="str">
-        <v>fail</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D7"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -987,7 +778,7 @@
         <v>SET_BASE_URL</v>
       </c>
       <c r="C2" t="str">
-        <v>https://justkept-dev.freewillsolutions.com</v>
+        <v>justkept-dev.freewillsolutions.com</v>
       </c>
     </row>
     <row r="3">
@@ -1040,7 +831,7 @@
         <v>LOG_RESPONSE</v>
       </c>
       <c r="C6" t="str">
-        <v>1500</v>
+        <v>500</v>
       </c>
     </row>
     <row r="7">
@@ -1057,93 +848,9 @@
         <v>pass</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8">
-        <v>7</v>
-      </c>
-      <c r="B8" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C8" t="str">
-        <v>messageCode|success</v>
-      </c>
-      <c r="D8" t="str">
-        <v>pass</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9">
-        <v>8</v>
-      </c>
-      <c r="B9" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C9" t="str">
-        <v>data.entity|notification</v>
-      </c>
-      <c r="D9" t="str">
-        <v>pass</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10">
-        <v>9</v>
-      </c>
-      <c r="B10" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C10" t="str">
-        <v>data.PK|9876543210987</v>
-      </c>
-      <c r="D10" t="str">
-        <v>pass</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11">
-        <v>10</v>
-      </c>
-      <c r="B11" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C11" t="str">
-        <v>data.status|SENT</v>
-      </c>
-      <c r="D11" t="str">
-        <v>pass</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12">
-        <v>11</v>
-      </c>
-      <c r="B12" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C12" t="str">
-        <v>data.customerId|9876543210987</v>
-      </c>
-      <c r="D12" t="str">
-        <v>pass</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13">
-        <v>12</v>
-      </c>
-      <c r="B13" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C13" t="str">
-        <v>data.notiChannel|On Web</v>
-      </c>
-      <c r="D13" t="str">
-        <v>pass</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D7"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1174,7 +881,7 @@
         <v>SET_BASE_URL</v>
       </c>
       <c r="C2" t="str">
-        <v>https://justkept-dev.freewillsolutions.com</v>
+        <v>justkept-dev.freewillsolutions.com</v>
       </c>
     </row>
     <row r="3">
@@ -1216,7 +923,7 @@
         <v>/api/s3/getobject</v>
       </c>
       <c r="D5" t="str">
-        <v>{"fileKey":"document/CUSTOMER/9876543210987/basic-text.pdf"}</v>
+        <v>{"fileKey":"document/CUSTOMER/9876543210987/JustKept_overview.drawio.pdf"}</v>
       </c>
     </row>
     <row r="6">
@@ -1227,7 +934,7 @@
         <v>LOG_RESPONSE</v>
       </c>
       <c r="C6" t="str">
-        <v>1500</v>
+        <v>500</v>
       </c>
     </row>
     <row r="7">
@@ -1253,7 +960,7 @@
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:D7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1277,7 +984,7 @@
         <v>SET_BASE_URL</v>
       </c>
       <c r="C2" t="str">
-        <v>https://justkept-dev.freewillsolutions.com</v>
+        <v>justkept-dev.freewillsolutions.com</v>
       </c>
     </row>
     <row r="3">
@@ -1319,7 +1026,7 @@
         <v>/api/broker/listuploaddraft</v>
       </c>
       <c r="D5" t="str">
-        <v>{"brokerId":"U1001","requestId":"fa00fc86-20e6-463f-8f98-6ad112107d9d"}</v>
+        <v>{"brokerId":"U1001","requestId":"REQ404"}</v>
       </c>
     </row>
     <row r="6">
@@ -1330,7 +1037,7 @@
         <v>LOG_RESPONSE</v>
       </c>
       <c r="C6" t="str">
-        <v>1500</v>
+        <v>500</v>
       </c>
     </row>
     <row r="7">
@@ -1347,156 +1054,16 @@
         <v>pass</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8">
-        <v>7</v>
-      </c>
-      <c r="B8" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C8" t="str">
-        <v>0.PK|U1001</v>
-      </c>
-      <c r="D8" t="str">
-        <v>pass</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9">
-        <v>8</v>
-      </c>
-      <c r="B9" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C9" t="str">
-        <v>0.entity|doc_draft</v>
-      </c>
-      <c r="D9" t="str">
-        <v>pass</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10">
-        <v>9</v>
-      </c>
-      <c r="B10" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C10" t="str">
-        <v>0.requestId|fa00fc86-20e6-463f-8f98-6ad112107d9d</v>
-      </c>
-      <c r="D10" t="str">
-        <v>pass</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11">
-        <v>10</v>
-      </c>
-      <c r="B11" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C11" t="str">
-        <v>0.customerId|undefined</v>
-      </c>
-      <c r="D11" t="str">
-        <v>fail</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12">
-        <v>11</v>
-      </c>
-      <c r="B12" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C12" t="str">
-        <v>0.createdAt|undefined</v>
-      </c>
-      <c r="D12" t="str">
-        <v>fail</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13">
-        <v>12</v>
-      </c>
-      <c r="B13" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C13" t="str">
-        <v>0.docType|undefined</v>
-      </c>
-      <c r="D13" t="str">
-        <v>fail</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14">
-        <v>13</v>
-      </c>
-      <c r="B14" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C14" t="str">
-        <v>0.draftId|undefined</v>
-      </c>
-      <c r="D14" t="str">
-        <v>fail</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15">
-        <v>14</v>
-      </c>
-      <c r="B15" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C15" t="str">
-        <v>0.emailTemplate|undefined</v>
-      </c>
-      <c r="D15" t="str">
-        <v>fail</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16">
-        <v>15</v>
-      </c>
-      <c r="B16" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C16" t="str">
-        <v>0.messageBody|undefined</v>
-      </c>
-      <c r="D16" t="str">
-        <v>fail</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17">
-        <v>16</v>
-      </c>
-      <c r="B17" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C17" t="str">
-        <v>0.subjectLine|undefined</v>
-      </c>
-      <c r="D17" t="str">
-        <v>fail</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D17"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D7"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1520,7 +1087,7 @@
         <v>SET_BASE_URL</v>
       </c>
       <c r="C2" t="str">
-        <v>https://justkept-dev.freewillsolutions.com</v>
+        <v>justkept-dev.freewillsolutions.com</v>
       </c>
     </row>
     <row r="3">
@@ -1573,7 +1140,7 @@
         <v>LOG_RESPONSE</v>
       </c>
       <c r="C6" t="str">
-        <v>1500</v>
+        <v>500</v>
       </c>
     </row>
     <row r="7">
@@ -1590,44 +1157,16 @@
         <v>pass</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8">
-        <v>7</v>
-      </c>
-      <c r="B8" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C8" t="str">
-        <v>messageCode|success</v>
-      </c>
-      <c r="D8" t="str">
-        <v>pass</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9">
-        <v>8</v>
-      </c>
-      <c r="B9" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C9" t="str">
-        <v>message|undefined</v>
-      </c>
-      <c r="D9" t="str">
-        <v>fail</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D7"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1651,7 +1190,7 @@
         <v>SET_BASE_URL</v>
       </c>
       <c r="C2" t="str">
-        <v>https://justkept-dev.freewillsolutions.com</v>
+        <v>justkept-dev.freewillsolutions.com</v>
       </c>
     </row>
     <row r="3">
@@ -1704,7 +1243,7 @@
         <v>LOG_RESPONSE</v>
       </c>
       <c r="C6" t="str">
-        <v>1500</v>
+        <v>500</v>
       </c>
     </row>
     <row r="7">
@@ -1721,58 +1260,16 @@
         <v>pass</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8">
-        <v>7</v>
-      </c>
-      <c r="B8" t="str">
-        <v>STORE_JSON</v>
-      </c>
-      <c r="C8" t="str">
-        <v>draftSK</v>
-      </c>
-      <c r="D8" t="str">
-        <v>draft_SK</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9">
-        <v>8</v>
-      </c>
-      <c r="B9" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C9" t="str">
-        <v>messageCode|success</v>
-      </c>
-      <c r="D9" t="str">
-        <v>pass</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10">
-        <v>9</v>
-      </c>
-      <c r="B10" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C10" t="str">
-        <v>message|undefined</v>
-      </c>
-      <c r="D10" t="str">
-        <v>fail</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D7"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D23"/>
+  <dimension ref="A1:D7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1796,7 +1293,7 @@
         <v>SET_BASE_URL</v>
       </c>
       <c r="C2" t="str">
-        <v>https://justkept-dev.freewillsolutions.com</v>
+        <v>justkept-dev.freewillsolutions.com</v>
       </c>
     </row>
     <row r="3">
@@ -1849,7 +1346,7 @@
         <v>LOG_RESPONSE</v>
       </c>
       <c r="C6" t="str">
-        <v>1500</v>
+        <v>500</v>
       </c>
     </row>
     <row r="7">
@@ -1866,233 +1363,9 @@
         <v>pass</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8">
-        <v>7</v>
-      </c>
-      <c r="B8" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C8" t="str">
-        <v>messageCode|success</v>
-      </c>
-      <c r="D8" t="str">
-        <v>pass</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9">
-        <v>8</v>
-      </c>
-      <c r="B9" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C9" t="str">
-        <v>message|undefined</v>
-      </c>
-      <c r="D9" t="str">
-        <v>fail</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10">
-        <v>9</v>
-      </c>
-      <c r="B10" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C10" t="str">
-        <v>data.entity|customer_req</v>
-      </c>
-      <c r="D10" t="str">
-        <v>pass</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11">
-        <v>10</v>
-      </c>
-      <c r="B11" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C11" t="str">
-        <v>data.customerId|9876543210987</v>
-      </c>
-      <c r="D11" t="str">
-        <v>pass</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12">
-        <v>11</v>
-      </c>
-      <c r="B12" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C12" t="str">
-        <v>data.requestId|2f70d0ec-f6f1-4ffb-aca3-fc93ea50749e</v>
-      </c>
-      <c r="D12" t="str">
-        <v>pass</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13">
-        <v>12</v>
-      </c>
-      <c r="B13" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C13" t="str">
-        <v>data.detail|undefined</v>
-      </c>
-      <c r="D13" t="str">
-        <v>fail</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14">
-        <v>13</v>
-      </c>
-      <c r="B14" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C14" t="str">
-        <v>data.fileNonRequiredPath|undefined</v>
-      </c>
-      <c r="D14" t="str">
-        <v>fail</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15">
-        <v>14</v>
-      </c>
-      <c r="B15" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C15" t="str">
-        <v>data.status|undefined</v>
-      </c>
-      <c r="D15" t="str">
-        <v>fail</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16">
-        <v>15</v>
-      </c>
-      <c r="B16" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C16" t="str">
-        <v>data.specifyDocType|undefined</v>
-      </c>
-      <c r="D16" t="str">
-        <v>fail</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17">
-        <v>16</v>
-      </c>
-      <c r="B17" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C17" t="str">
-        <v>data.requestTopic|undefined</v>
-      </c>
-      <c r="D17" t="str">
-        <v>fail</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18">
-        <v>17</v>
-      </c>
-      <c r="B18" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C18" t="str">
-        <v>data.subCompanyId|undefined</v>
-      </c>
-      <c r="D18" t="str">
-        <v>fail</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19">
-        <v>18</v>
-      </c>
-      <c r="B19" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C19" t="str">
-        <v>data.isDraft|undefined</v>
-      </c>
-      <c r="D19" t="str">
-        <v>fail</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20">
-        <v>19</v>
-      </c>
-      <c r="B20" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C20" t="str">
-        <v>data.subCompanyId|undefined</v>
-      </c>
-      <c r="D20" t="str">
-        <v>fail</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21">
-        <v>20</v>
-      </c>
-      <c r="B21" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C21" t="str">
-        <v>data.requestType|undefined</v>
-      </c>
-      <c r="D21" t="str">
-        <v>fail</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22">
-        <v>21</v>
-      </c>
-      <c r="B22" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C22" t="str">
-        <v>data.updatedAt|undefined</v>
-      </c>
-      <c r="D22" t="str">
-        <v>fail</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23">
-        <v>22</v>
-      </c>
-      <c r="B23" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C23" t="str">
-        <v>data.fileRequiredPath|undefined</v>
-      </c>
-      <c r="D23" t="str">
-        <v>fail</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D23"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D7"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2123,7 +1396,7 @@
         <v>SET_BASE_URL</v>
       </c>
       <c r="C2" t="str">
-        <v>https://justkept-dev.freewillsolutions.com</v>
+        <v>justkept-dev.freewillsolutions.com</v>
       </c>
     </row>
     <row r="3">
@@ -2165,7 +1438,7 @@
         <v>/api/broker/listscheduledraft</v>
       </c>
       <c r="D5" t="str">
-        <v>{"brokerId":"U1001"}</v>
+        <v>{"brokerId":"0105566000888"}</v>
       </c>
     </row>
     <row r="6">
@@ -2176,7 +1449,7 @@
         <v>LOG_RESPONSE</v>
       </c>
       <c r="C6" t="str">
-        <v>1500</v>
+        <v>500</v>
       </c>
     </row>
     <row r="7">
@@ -2202,7 +1475,7 @@
 
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2226,7 +1499,7 @@
         <v>SET_BASE_URL</v>
       </c>
       <c r="C2" t="str">
-        <v>https://justkept-dev.freewillsolutions.com</v>
+        <v>justkept-dev.freewillsolutions.com</v>
       </c>
     </row>
     <row r="3">
@@ -2265,10 +1538,10 @@
         <v>API_POST</v>
       </c>
       <c r="C5" t="str">
-        <v>/api/broker/customerlogs</v>
+        <v>/api/audit/findauditlogs</v>
       </c>
       <c r="D5" t="str">
-        <v>{"customerId":"9876543210987"}</v>
+        <v>{"actorId":"9876543210987","actorRole":"CUSTOMER"}</v>
       </c>
     </row>
     <row r="6">
@@ -2279,7 +1552,7 @@
         <v>LOG_RESPONSE</v>
       </c>
       <c r="C6" t="str">
-        <v>1500</v>
+        <v>500</v>
       </c>
     </row>
     <row r="7">
@@ -2296,114 +1569,16 @@
         <v>pass</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8">
-        <v>7</v>
-      </c>
-      <c r="B8" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C8" t="str">
-        <v>0.actorId|9876543210987</v>
-      </c>
-      <c r="D8" t="str">
-        <v>pass</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9">
-        <v>8</v>
-      </c>
-      <c r="B9" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C9" t="str">
-        <v>0.entity|audit_log</v>
-      </c>
-      <c r="D9" t="str">
-        <v>pass</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10">
-        <v>9</v>
-      </c>
-      <c r="B10" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C10" t="str">
-        <v>0.targetId|undefined</v>
-      </c>
-      <c r="D10" t="str">
-        <v>fail</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11">
-        <v>10</v>
-      </c>
-      <c r="B11" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C11" t="str">
-        <v>0.auditId|undefined</v>
-      </c>
-      <c r="D11" t="str">
-        <v>fail</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12">
-        <v>11</v>
-      </c>
-      <c r="B12" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C12" t="str">
-        <v>0.actorId|undefined</v>
-      </c>
-      <c r="D12" t="str">
-        <v>fail</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13">
-        <v>12</v>
-      </c>
-      <c r="B13" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C13" t="str">
-        <v>0.actorRole|undefined</v>
-      </c>
-      <c r="D13" t="str">
-        <v>fail</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14">
-        <v>13</v>
-      </c>
-      <c r="B14" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C14" t="str">
-        <v>0.action|undefined</v>
-      </c>
-      <c r="D14" t="str">
-        <v>fail</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D14"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D7"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2427,7 +1602,7 @@
         <v>SET_BASE_URL</v>
       </c>
       <c r="C2" t="str">
-        <v>https://justkept-dev.freewillsolutions.com</v>
+        <v>justkept-dev.freewillsolutions.com</v>
       </c>
     </row>
     <row r="3">
@@ -2497,30 +1672,16 @@
         <v>pass</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8">
-        <v>7</v>
-      </c>
-      <c r="B8" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C8" t="str">
-        <v>0.PK|9876543210987</v>
-      </c>
-      <c r="D8" t="str">
-        <v>pass</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D7"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:D7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2544,7 +1705,7 @@
         <v>SET_BASE_URL</v>
       </c>
       <c r="C2" t="str">
-        <v>https://justkept-dev.freewillsolutions.com</v>
+        <v>justkept-dev.freewillsolutions.com</v>
       </c>
     </row>
     <row r="3">
@@ -2583,10 +1744,10 @@
         <v>API_POST</v>
       </c>
       <c r="C5" t="str">
-        <v>/api/broker/findallcustomerbysubcomid</v>
+        <v>/api/broker/customerlogs</v>
       </c>
       <c r="D5" t="str">
-        <v>{"brokerId":"U1001"}</v>
+        <v>{"customerId":"9876543210987"}</v>
       </c>
     </row>
     <row r="6">
@@ -2597,7 +1758,7 @@
         <v>LOG_RESPONSE</v>
       </c>
       <c r="C6" t="str">
-        <v>1500</v>
+        <v>500</v>
       </c>
     </row>
     <row r="7">
@@ -2614,156 +1775,119 @@
         <v>pass</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8">
-        <v>7</v>
-      </c>
-      <c r="B8" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C8" t="str">
-        <v>0.entity|relationship</v>
-      </c>
-      <c r="D8" t="str">
-        <v>pass</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9">
-        <v>8</v>
-      </c>
-      <c r="B9" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C9" t="str">
-        <v>0.PK|customer_relationship</v>
-      </c>
-      <c r="D9" t="str">
-        <v>pass</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10">
-        <v>9</v>
-      </c>
-      <c r="B10" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C10" t="str">
-        <v>0.customerName|undefined</v>
-      </c>
-      <c r="D10" t="str">
-        <v>fail</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11">
-        <v>10</v>
-      </c>
-      <c r="B11" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C11" t="str">
-        <v>0.ID_Number|undefined</v>
-      </c>
-      <c r="D11" t="str">
-        <v>fail</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12">
-        <v>11</v>
-      </c>
-      <c r="B12" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C12" t="str">
-        <v>0.subCompanyId|undefined</v>
-      </c>
-      <c r="D12" t="str">
-        <v>fail</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13">
-        <v>12</v>
-      </c>
-      <c r="B13" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C13" t="str">
-        <v>0.status|undefined</v>
-      </c>
-      <c r="D13" t="str">
-        <v>fail</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14">
-        <v>13</v>
-      </c>
-      <c r="B14" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C14" t="str">
-        <v>0.pendingReq|undefined</v>
-      </c>
-      <c r="D14" t="str">
-        <v>fail</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15">
-        <v>14</v>
-      </c>
-      <c r="B15" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C15" t="str">
-        <v>0.totalDocuments|undefined</v>
-      </c>
-      <c r="D15" t="str">
-        <v>fail</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16">
-        <v>15</v>
-      </c>
-      <c r="B16" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C16" t="str">
-        <v>0.email|undefined</v>
-      </c>
-      <c r="D16" t="str">
-        <v>fail</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17">
-        <v>16</v>
-      </c>
-      <c r="B17" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C17" t="str">
-        <v>0.customerIdGSIPK|undefined</v>
-      </c>
-      <c r="D17" t="str">
-        <v>fail</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D17"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D7"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D7"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Step</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Action</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Target</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Data</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="str">
+        <v>SET_BASE_URL</v>
+      </c>
+      <c r="C2" t="str">
+        <v>justkept-dev.freewillsolutions.com</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="str">
+        <v>SET_HEADER</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Content-Type</v>
+      </c>
+      <c r="D3" t="str">
+        <v>application/json</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="str">
+        <v>SET_HEADER</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Authorization</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Bearer {{ACCESS_TOKEN}}</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="str">
+        <v>API_POST</v>
+      </c>
+      <c r="C5" t="str">
+        <v>/api/broker/findallcustomerbysubcomid</v>
+      </c>
+      <c r="D5" t="str">
+        <v>{"brokerId":"U1001"}</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="str">
+        <v>LOG_RESPONSE</v>
+      </c>
+      <c r="C6" t="str">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="str">
+        <v>CHECK_STATUS</v>
+      </c>
+      <c r="C7" t="str">
+        <v>200</v>
+      </c>
+      <c r="D7" t="str">
+        <v>pass</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:D7"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2787,7 +1911,7 @@
         <v>SET_BASE_URL</v>
       </c>
       <c r="C2" t="str">
-        <v>https://justkept-dev.freewillsolutions.com</v>
+        <v>justkept-dev.freewillsolutions.com</v>
       </c>
     </row>
     <row r="3">
@@ -2857,30 +1981,16 @@
         <v>pass</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8">
-        <v>7</v>
-      </c>
-      <c r="B8" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C8" t="str">
-        <v>data.length|0</v>
-      </c>
-      <c r="D8" t="str">
-        <v>fail</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D7"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2904,7 +2014,7 @@
         <v>SET_BASE_URL</v>
       </c>
       <c r="C2" t="str">
-        <v>https://justkept-dev.freewillsolutions.com</v>
+        <v>justkept-dev.freewillsolutions.com</v>
       </c>
     </row>
     <row r="3">
@@ -2974,72 +2084,16 @@
         <v>pass</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8">
-        <v>7</v>
-      </c>
-      <c r="B8" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C8" t="str">
-        <v>0.PK|9876543210987</v>
-      </c>
-      <c r="D8" t="str">
-        <v>pass</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9">
-        <v>8</v>
-      </c>
-      <c r="B9" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C9" t="str">
-        <v>0.entity|customer_req</v>
-      </c>
-      <c r="D9" t="str">
-        <v>pass</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10">
-        <v>9</v>
-      </c>
-      <c r="B10" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C10" t="str">
-        <v>0.requestId|undefined</v>
-      </c>
-      <c r="D10" t="str">
-        <v>fail</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11">
-        <v>10</v>
-      </c>
-      <c r="B11" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C11" t="str">
-        <v>0.subCompanyId|undefined</v>
-      </c>
-      <c r="D11" t="str">
-        <v>fail</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D7"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -3063,7 +2117,7 @@
         <v>SET_BASE_URL</v>
       </c>
       <c r="C2" t="str">
-        <v>https://justkept-dev.freewillsolutions.com</v>
+        <v>justkept-dev.freewillsolutions.com</v>
       </c>
     </row>
     <row r="3">
@@ -3116,7 +2170,7 @@
         <v>LOG_RESPONSE</v>
       </c>
       <c r="C6" t="str">
-        <v>1500</v>
+        <v>500</v>
       </c>
     </row>
     <row r="7">
@@ -3133,128 +2187,16 @@
         <v>pass</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8">
-        <v>7</v>
-      </c>
-      <c r="B8" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C8" t="str">
-        <v>data.0.PK|9876543210987</v>
-      </c>
-      <c r="D8" t="str">
-        <v>pass</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9">
-        <v>8</v>
-      </c>
-      <c r="B9" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C9" t="str">
-        <v>data.0.sourceSystem|BROKER_MANUAL_UPLOAD</v>
-      </c>
-      <c r="D9" t="str">
-        <v>pass</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10">
-        <v>9</v>
-      </c>
-      <c r="B10" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C10" t="str">
-        <v>data.0.fileName|undefined</v>
-      </c>
-      <c r="D10" t="str">
-        <v>fail</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11">
-        <v>10</v>
-      </c>
-      <c r="B11" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C11" t="str">
-        <v>data.0.requestId|undefined</v>
-      </c>
-      <c r="D11" t="str">
-        <v>fail</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12">
-        <v>11</v>
-      </c>
-      <c r="B12" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C12" t="str">
-        <v>data.0.filePath|undefined</v>
-      </c>
-      <c r="D12" t="str">
-        <v>fail</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13">
-        <v>12</v>
-      </c>
-      <c r="B13" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C13" t="str">
-        <v>data.0.docType|undefined</v>
-      </c>
-      <c r="D13" t="str">
-        <v>fail</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14">
-        <v>13</v>
-      </c>
-      <c r="B14" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C14" t="str">
-        <v>data.0.docId|undefined</v>
-      </c>
-      <c r="D14" t="str">
-        <v>fail</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15">
-        <v>14</v>
-      </c>
-      <c r="B15" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C15" t="str">
-        <v>data.0.SK_SORT|undefined</v>
-      </c>
-      <c r="D15" t="str">
-        <v>fail</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D15"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D7"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -3278,7 +2220,7 @@
         <v>SET_BASE_URL</v>
       </c>
       <c r="C2" t="str">
-        <v>https://justkept-dev.freewillsolutions.com</v>
+        <v>justkept-dev.freewillsolutions.com</v>
       </c>
     </row>
     <row r="3">
@@ -3331,7 +2273,7 @@
         <v>LOG_RESPONSE</v>
       </c>
       <c r="C6" t="str">
-        <v>5500</v>
+        <v>500</v>
       </c>
     </row>
     <row r="7">
@@ -3348,72 +2290,16 @@
         <v>pass</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8">
-        <v>7</v>
-      </c>
-      <c r="B8" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C8" t="str">
-        <v>0.entity|req_topic</v>
-      </c>
-      <c r="D8" t="str">
-        <v>pass</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9">
-        <v>8</v>
-      </c>
-      <c r="B9" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C9" t="str">
-        <v>0.PK|BKK01</v>
-      </c>
-      <c r="D9" t="str">
-        <v>pass</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10">
-        <v>9</v>
-      </c>
-      <c r="B10" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C10" t="str">
-        <v>0.req_topic_id|undefined</v>
-      </c>
-      <c r="D10" t="str">
-        <v>fail</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11">
-        <v>10</v>
-      </c>
-      <c r="B11" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C11" t="str">
-        <v>0.config|undefined</v>
-      </c>
-      <c r="D11" t="str">
-        <v>fail</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D7"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -3437,7 +2323,7 @@
         <v>SET_BASE_URL</v>
       </c>
       <c r="C2" t="str">
-        <v>https://justkept-dev.freewillsolutions.com</v>
+        <v>justkept-dev.freewillsolutions.com</v>
       </c>
     </row>
     <row r="3">
@@ -3490,7 +2376,7 @@
         <v>LOG_RESPONSE</v>
       </c>
       <c r="C6" t="str">
-        <v>1500</v>
+        <v>500</v>
       </c>
     </row>
     <row r="7">
@@ -3507,72 +2393,16 @@
         <v>pass</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8">
-        <v>7</v>
-      </c>
-      <c r="B8" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C8" t="str">
-        <v>data.0.PK|9876543210987</v>
-      </c>
-      <c r="D8" t="str">
-        <v>pass</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9">
-        <v>8</v>
-      </c>
-      <c r="B9" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C9" t="str">
-        <v>data.0.entity|notification</v>
-      </c>
-      <c r="D9" t="str">
-        <v>pass</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10">
-        <v>9</v>
-      </c>
-      <c r="B10" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C10" t="str">
-        <v>data.0.isRead|undefined</v>
-      </c>
-      <c r="D10" t="str">
-        <v>fail</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11">
-        <v>10</v>
-      </c>
-      <c r="B11" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C11" t="str">
-        <v>data.0.title|undefined</v>
-      </c>
-      <c r="D11" t="str">
-        <v>fail</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D7"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -3596,7 +2426,7 @@
         <v>SET_BASE_URL</v>
       </c>
       <c r="C2" t="str">
-        <v>https://justkept-dev.freewillsolutions.com</v>
+        <v>justkept-dev.freewillsolutions.com</v>
       </c>
     </row>
     <row r="3">
@@ -3649,7 +2479,7 @@
         <v>LOG_RESPONSE</v>
       </c>
       <c r="C6" t="str">
-        <v>1500</v>
+        <v>500</v>
       </c>
     </row>
     <row r="7">
@@ -3666,86 +2496,16 @@
         <v>pass</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8">
-        <v>7</v>
-      </c>
-      <c r="B8" t="str">
-        <v>STORE_JSON</v>
-      </c>
-      <c r="C8" t="str">
-        <v>result.0.requestId</v>
-      </c>
-      <c r="D8" t="str">
-        <v>REQUEST_ID</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9">
-        <v>8</v>
-      </c>
-      <c r="B9" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C9" t="str">
-        <v>result.0.customerId|9876543210987</v>
-      </c>
-      <c r="D9" t="str">
-        <v>pass</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10">
-        <v>9</v>
-      </c>
-      <c r="B10" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C10" t="str">
-        <v>result.0.entity|doc_metadata</v>
-      </c>
-      <c r="D10" t="str">
-        <v>pass</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11">
-        <v>10</v>
-      </c>
-      <c r="B11" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C11" t="str">
-        <v>result.0.SK_SORT|undefined</v>
-      </c>
-      <c r="D11" t="str">
-        <v>fail</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12">
-        <v>11</v>
-      </c>
-      <c r="B12" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C12" t="str">
-        <v>result.0.requestId|undefined</v>
-      </c>
-      <c r="D12" t="str">
-        <v>fail</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D12"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D7"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D26"/>
+  <dimension ref="A1:D7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -3769,7 +2529,7 @@
         <v>SET_BASE_URL</v>
       </c>
       <c r="C2" t="str">
-        <v>https://justkept-dev.freewillsolutions.com</v>
+        <v>justkept-dev.freewillsolutions.com</v>
       </c>
     </row>
     <row r="3">
@@ -3811,7 +2571,7 @@
         <v>/api/broker/findschedules</v>
       </c>
       <c r="D5" t="str">
-        <v>{"brokerId":"U1001"}</v>
+        <v>{"brokerId":"0105566000888"}</v>
       </c>
     </row>
     <row r="6">
@@ -3822,7 +2582,7 @@
         <v>LOG_RESPONSE</v>
       </c>
       <c r="C6" t="str">
-        <v>1500</v>
+        <v>500</v>
       </c>
     </row>
     <row r="7">
@@ -3839,275 +2599,9 @@
         <v>pass</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8">
-        <v>7</v>
-      </c>
-      <c r="B8" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C8" t="str">
-        <v>items.0.brokerId|U1001</v>
-      </c>
-      <c r="D8" t="str">
-        <v>pass</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9">
-        <v>8</v>
-      </c>
-      <c r="B9" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C9" t="str">
-        <v>items.0.PK|BKK01</v>
-      </c>
-      <c r="D9" t="str">
-        <v>pass</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10">
-        <v>9</v>
-      </c>
-      <c r="B10" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C10" t="str">
-        <v>items.0.entity|system_schedule_job</v>
-      </c>
-      <c r="D10" t="str">
-        <v>pass</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11">
-        <v>10</v>
-      </c>
-      <c r="B11" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C11" t="str">
-        <v>items.0.recipientCount|undefined</v>
-      </c>
-      <c r="D11" t="str">
-        <v>fail</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12">
-        <v>11</v>
-      </c>
-      <c r="B12" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C12" t="str">
-        <v>items.0.secretKey|undefined</v>
-      </c>
-      <c r="D12" t="str">
-        <v>fail</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13">
-        <v>12</v>
-      </c>
-      <c r="B13" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C13" t="str">
-        <v>items.0.subject|undefined</v>
-      </c>
-      <c r="D13" t="str">
-        <v>fail</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14">
-        <v>13</v>
-      </c>
-      <c r="B14" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C14" t="str">
-        <v>items.0.runAt|undefined</v>
-      </c>
-      <c r="D14" t="str">
-        <v>fail</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15">
-        <v>14</v>
-      </c>
-      <c r="B15" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C15" t="str">
-        <v>items.0.nextRunAt|undefined</v>
-      </c>
-      <c r="D15" t="str">
-        <v>fail</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16">
-        <v>15</v>
-      </c>
-      <c r="B16" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C16" t="str">
-        <v>items.0.stopAt|undefined</v>
-      </c>
-      <c r="D16" t="str">
-        <v>fail</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17">
-        <v>16</v>
-      </c>
-      <c r="B17" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C17" t="str">
-        <v>items.0.secretName|undefined</v>
-      </c>
-      <c r="D17" t="str">
-        <v>fail</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18">
-        <v>17</v>
-      </c>
-      <c r="B18" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C18" t="str">
-        <v>items.0.createdAt|undefined</v>
-      </c>
-      <c r="D18" t="str">
-        <v>fail</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19">
-        <v>18</v>
-      </c>
-      <c r="B19" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C19" t="str">
-        <v>items.0.sourceType|undefined</v>
-      </c>
-      <c r="D19" t="str">
-        <v>fail</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20">
-        <v>19</v>
-      </c>
-      <c r="B20" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C20" t="str">
-        <v>items.0.sourcePath|undefined</v>
-      </c>
-      <c r="D20" t="str">
-        <v>fail</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21">
-        <v>20</v>
-      </c>
-      <c r="B21" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C21" t="str">
-        <v>items.0.frequency|undefined</v>
-      </c>
-      <c r="D21" t="str">
-        <v>fail</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22">
-        <v>21</v>
-      </c>
-      <c r="B22" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C22" t="str">
-        <v>items.0.jobId|undefined</v>
-      </c>
-      <c r="D22" t="str">
-        <v>fail</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23">
-        <v>22</v>
-      </c>
-      <c r="B23" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C23" t="str">
-        <v>items.0.docType|undefined</v>
-      </c>
-      <c r="D23" t="str">
-        <v>fail</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24">
-        <v>23</v>
-      </c>
-      <c r="B24" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C24" t="str">
-        <v>items.0.dayOfMonth|undefined</v>
-      </c>
-      <c r="D24" t="str">
-        <v>fail</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25">
-        <v>24</v>
-      </c>
-      <c r="B25" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C25" t="str">
-        <v>items.0.displayRecipientName|undefined</v>
-      </c>
-      <c r="D25" t="str">
-        <v>fail</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26">
-        <v>25</v>
-      </c>
-      <c r="B26" t="str">
-        <v>CHECK_JSON</v>
-      </c>
-      <c r="C26" t="str">
-        <v>items.0.jobStatus|undefined</v>
-      </c>
-      <c r="D26" t="str">
-        <v>fail</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D26"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D7"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>